<commit_message>
Document PD model testing and historical limitation
</commit_message>
<xml_diff>
--- a/docs/eit/exception_log.xlsx
+++ b/docs/eit/exception_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub Projects\freddie-mac-credit-risk\docs\eit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D74A3F76-DFCD-49CD-9A46-3614F362909C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91A3AA6B-08DC-4CBB-A0F1-CD06FD379C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="18648" windowHeight="11784" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="107">
   <si>
     <t>Mortgage Data and Credit-Risk Reporting — Exception Log</t>
   </si>
@@ -325,6 +325,36 @@
   </si>
   <si>
     <t>Data exceptions</t>
+  </si>
+  <si>
+    <t>L-03</t>
+  </si>
+  <si>
+    <t>EIT-14; EIT-15</t>
+  </si>
+  <si>
+    <t>Historical channel level unavailable in development</t>
+  </si>
+  <si>
+    <t>The 2006 historical population contained channel T for 22,031 of 37,555 eligible loans (58.66%). Channel T was absent from the 2015–2016 development population and was treated as an unknown category during scoring.</t>
+  </si>
+  <si>
+    <t>Scoring categories should be represented in development data or processed through a controlled unknown-category treatment with documented limitations.</t>
+  </si>
+  <si>
+    <t>Channel distributions changed across vintages. Channel T was present in 2006 but absent from the selected 2015–2016 development population. The configured encoder safely ignored the unknown level during scoring.</t>
+  </si>
+  <si>
+    <t>The model cannot separately estimate the effect of channel T. Historical 2006 calibration and discrimination may therefore be influenced. The primary 2017 final-test population was not affected.</t>
+  </si>
+  <si>
+    <t>Restrict the 2006 results to historical sensitivity analysis, document the unknown-category limitation, and monitor unknown categorical levels before any future model use.</t>
+  </si>
+  <si>
+    <t>05_pd_modeling.ipynb — unknown-category audit; data/processed/unknown_category_audit.csv; docs/eit/07_pd_model_testing_workpaper.md</t>
+  </si>
+  <si>
+    <t>Closed — The affected population was quantified and isolated to the 2006 historical comparison. The primary 2017 test contained zero unknown categories. Historical use was restricted and the limitation was documented.</t>
   </si>
 </sst>
 </file>
@@ -589,44 +619,44 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -951,7 +981,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -972,64 +1002,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="30" customHeight="1">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16"/>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="P1" s="16"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
     </row>
     <row r="2" spans="1:16" ht="14.4">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="17"/>
-      <c r="M2" s="17"/>
-      <c r="N2" s="17"/>
-      <c r="O2" s="17"/>
-      <c r="P2" s="17"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
+      <c r="L2" s="29"/>
+      <c r="M2" s="29"/>
+      <c r="N2" s="29"/>
+      <c r="O2" s="29"/>
+      <c r="P2" s="29"/>
     </row>
     <row r="3" spans="1:16">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
-      <c r="N3" s="18"/>
-      <c r="O3" s="18"/>
-      <c r="P3" s="18"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
+      <c r="K3" s="30"/>
+      <c r="L3" s="30"/>
+      <c r="M3" s="30"/>
+      <c r="N3" s="30"/>
+      <c r="O3" s="30"/>
+      <c r="P3" s="30"/>
     </row>
     <row r="5" spans="1:16" ht="42" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -1327,6 +1357,56 @@
       </c>
       <c r="P10" s="4" t="s">
         <v>95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="124.95" customHeight="1">
+      <c r="A11" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="10">
+        <v>46254</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="N11" s="10">
+        <v>46254</v>
+      </c>
+      <c r="O11" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="P11" s="4" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -1398,16 +1478,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
     </row>
     <row r="2" spans="1:8" ht="14.4">
       <c r="A2" s="11"/>
@@ -1420,15 +1500,15 @@
       <c r="H2" s="11"/>
     </row>
     <row r="3" spans="1:8" ht="14.4">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="B3" s="20"/>
+      <c r="B3" s="26"/>
       <c r="C3" s="11"/>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="E3" s="20"/>
+      <c r="E3" s="26"/>
       <c r="F3" s="11"/>
       <c r="G3" s="11"/>
       <c r="H3" s="11"/>
@@ -1439,7 +1519,7 @@
       </c>
       <c r="B4" s="13">
         <f>COUNTA('Exception Log'!$A$6:$A$30)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="12" t="s">
@@ -1447,7 +1527,7 @@
       </c>
       <c r="E4" s="13">
         <f>COUNTIF('Exception Log'!$C$6:$C$30,"Low")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F4" s="11"/>
       <c r="G4" s="11"/>
@@ -1499,7 +1579,7 @@
       </c>
       <c r="B7" s="13">
         <f>COUNTIF('Exception Log'!$D$6:$D$30,"Closed")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7" s="11"/>
       <c r="D7" s="12" t="s">
@@ -1534,7 +1614,7 @@
       </c>
       <c r="B9" s="13">
         <f>COUNTIF('Exception Log'!$B$6:$B$30,"Scope Limitation")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C9" s="11"/>
       <c r="D9" s="11"/>
@@ -1559,16 +1639,16 @@
       <c r="H10" s="11"/>
     </row>
     <row r="11" spans="1:8" ht="14.4">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="B11" s="21"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="21"/>
-      <c r="H11" s="21"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
     </row>
     <row r="12" spans="1:8" ht="14.4">
       <c r="A12" s="14" t="s">
@@ -1661,58 +1741,58 @@
       <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" ht="14.4">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="21"/>
+      <c r="B18" s="27"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
     </row>
     <row r="19" spans="1:8" ht="25.95" customHeight="1">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="24"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="18"/>
     </row>
     <row r="20" spans="1:8" ht="25.95" customHeight="1">
-      <c r="A20" s="25"/>
-      <c r="B20" s="26"/>
-      <c r="C20" s="26"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-      <c r="H20" s="27"/>
+      <c r="A20" s="19"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="21"/>
     </row>
     <row r="21" spans="1:8" ht="25.95" customHeight="1">
-      <c r="A21" s="25"/>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26"/>
-      <c r="H21" s="27"/>
+      <c r="A21" s="19"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="21"/>
     </row>
     <row r="22" spans="1:8" ht="25.95" customHeight="1">
-      <c r="A22" s="28"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="29"/>
-      <c r="G22" s="29"/>
-      <c r="H22" s="30"/>
+      <c r="A22" s="22"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>